<commit_message>
feat: add recharts library and implement various charts in Results component for enhanced data visualization
</commit_message>
<xml_diff>
--- a/data/database/metrics.xlsx
+++ b/data/database/metrics.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Resultados por Pregunta SIMCE</t>
+          <t>Resultados SIMCE por Pregunta</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -507,7 +507,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-02 15:20:17</t>
+          <t>2026-03-10 15:21:48</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">

</xml_diff>

<commit_message>
feat: add data processing and visualization enhancements, including new ETL logic and updated Results component
</commit_message>
<xml_diff>
--- a/data/database/metrics.xlsx
+++ b/data/database/metrics.xlsx
@@ -507,12 +507,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-10 15:21:48</t>
+          <t>2026-03-10 15:40:39</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{"fields": [{"name": "A", "type": "float"}, {"name": "B", "type": "float"}, {"name": "C", "type": "float"}, {"name": "D", "type": "float"}, {"name": "E", "type": "float"}, {"name": "Correcta", "type": "str"}, {"name": "Distractor", "type": "str"}]}</t>
+          <t>{"fields": [{"name": "A", "type": "float"}, {"name": "B", "type": "float"}, {"name": "C", "type": "float"}, {"name": "D", "type": "float"}, {"name": "E", "type": "float"}, {"name": "Correcta", "type": "str"}, {"name": "Distractor", "type": "str"}, {"name": "Rend", "type": "float"}]}</t>
         </is>
       </c>
     </row>

</xml_diff>